<commit_message>
Updating obsv file for treading damage simulation
</commit_message>
<xml_diff>
--- a/Tests/Validation/System/TreadingDamage/TreadingDamageTestOBS.xlsx
+++ b/Tests/Validation/System/TreadingDamage/TreadingDamageTestOBS.xlsx
@@ -1,21 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\aaUnderVC\ApsimX\Tests\Validation\System\TreadingDamage\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ApsimX\Tests\Validation\System\TreadingDamage\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{72FB3584-068C-4EB3-8213-A00DECC2D988}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D43760E7-3782-4188-8A3D-0E444C7FF165}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13680" yWindow="3750" windowWidth="29760" windowHeight="15885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Benchmark" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -129,8 +142,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -435,6 +449,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="8" max="8" width="10.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -490,14 +507,14 @@
       <c r="G2" t="s">
         <v>14</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="1">
         <v>37802</v>
       </c>
       <c r="I2">
         <v>0</v>
       </c>
       <c r="J2">
-        <v>47185.026275073498</v>
+        <v>38801.194000000003</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -522,14 +539,14 @@
       <c r="G3" t="s">
         <v>14</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="1">
         <v>37802</v>
       </c>
       <c r="I3">
         <v>1000</v>
       </c>
       <c r="J3">
-        <v>40401.505449555101</v>
+        <v>33723.942000000003</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -554,14 +571,14 @@
       <c r="G4" t="s">
         <v>14</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="1">
         <v>37802</v>
       </c>
       <c r="I4">
         <v>1500</v>
       </c>
       <c r="J4">
-        <v>39043.972404638298</v>
+        <v>33065.756999999998</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -586,14 +603,14 @@
       <c r="G5" t="s">
         <v>14</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="1">
         <v>37802</v>
       </c>
       <c r="I5">
         <v>250</v>
       </c>
       <c r="J5">
-        <v>44003.387970832002</v>
+        <v>35183.129999999997</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -618,14 +635,14 @@
       <c r="G6" t="s">
         <v>14</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="1">
         <v>37802</v>
       </c>
       <c r="I6">
         <v>500</v>
       </c>
       <c r="J6">
-        <v>42307.043826282897</v>
+        <v>34596.44</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -650,14 +667,14 @@
       <c r="G7" t="s">
         <v>14</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="1">
         <v>37802</v>
       </c>
       <c r="I7">
         <v>750</v>
       </c>
       <c r="J7">
-        <v>41193.622039403403</v>
+        <v>34145.279000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updating obs file for the TreadingDamage simualtion
</commit_message>
<xml_diff>
--- a/Tests/Validation/System/TreadingDamage/TreadingDamageTestOBS.xlsx
+++ b/Tests/Validation/System/TreadingDamage/TreadingDamageTestOBS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ApsimX\Tests\Validation\System\TreadingDamage\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D43760E7-3782-4188-8A3D-0E444C7FF165}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F659BF56-0E69-4262-A316-DED0CBBF65D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -514,7 +514,7 @@
         <v>0</v>
       </c>
       <c r="J2">
-        <v>38801.194000000003</v>
+        <v>40392.400000000001</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -546,7 +546,7 @@
         <v>1000</v>
       </c>
       <c r="J3">
-        <v>33723.942000000003</v>
+        <v>38627.599999999999</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -578,7 +578,7 @@
         <v>1500</v>
       </c>
       <c r="J4">
-        <v>33065.756999999998</v>
+        <v>37927.800000000003</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -610,7 +610,7 @@
         <v>250</v>
       </c>
       <c r="J5">
-        <v>35183.129999999997</v>
+        <v>39842</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -642,7 +642,7 @@
         <v>500</v>
       </c>
       <c r="J6">
-        <v>34596.44</v>
+        <v>39473.800000000003</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -674,7 +674,7 @@
         <v>750</v>
       </c>
       <c r="J7">
-        <v>34145.279000000002</v>
+        <v>39035.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>